<commit_message>
Standardize workflow names and configurations for 100% CI pass rate
</commit_message>
<xml_diff>
--- a/Test Results/Excel/Passed_Test_Cases.xlsx
+++ b/Test Results/Excel/Passed_Test_Cases.xlsx
@@ -480,7 +480,7 @@
         </is>
       </c>
       <c r="F2" t="n">
-        <v>0.19</v>
+        <v>0.21</v>
       </c>
       <c r="G2" t="inlineStr"/>
     </row>
@@ -511,7 +511,7 @@
         </is>
       </c>
       <c r="F3" t="n">
-        <v>0.2</v>
+        <v>0.19</v>
       </c>
       <c r="G3" t="inlineStr"/>
     </row>
@@ -573,7 +573,7 @@
         </is>
       </c>
       <c r="F5" t="n">
-        <v>0.18</v>
+        <v>0.23</v>
       </c>
       <c r="G5" t="inlineStr"/>
     </row>
@@ -604,7 +604,7 @@
         </is>
       </c>
       <c r="F6" t="n">
-        <v>0.25</v>
+        <v>0.23</v>
       </c>
       <c r="G6" t="inlineStr"/>
     </row>
@@ -635,7 +635,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.17</v>
       </c>
       <c r="G7" t="inlineStr"/>
     </row>
@@ -666,7 +666,7 @@
         </is>
       </c>
       <c r="F8" t="n">
-        <v>0.11</v>
+        <v>0.23</v>
       </c>
       <c r="G8" t="inlineStr"/>
     </row>
@@ -697,7 +697,7 @@
         </is>
       </c>
       <c r="F9" t="n">
-        <v>0.06</v>
+        <v>0.16</v>
       </c>
       <c r="G9" t="inlineStr"/>
     </row>
@@ -728,7 +728,7 @@
         </is>
       </c>
       <c r="F10" t="n">
-        <v>0.21</v>
+        <v>0.13</v>
       </c>
       <c r="G10" t="inlineStr"/>
     </row>
@@ -759,7 +759,7 @@
         </is>
       </c>
       <c r="F11" t="n">
-        <v>0.12</v>
+        <v>0.2</v>
       </c>
       <c r="G11" t="inlineStr"/>
     </row>
@@ -790,7 +790,7 @@
         </is>
       </c>
       <c r="F12" t="n">
-        <v>0.08</v>
+        <v>0.18</v>
       </c>
       <c r="G12" t="inlineStr"/>
     </row>
@@ -852,7 +852,7 @@
         </is>
       </c>
       <c r="F14" t="n">
-        <v>0.11</v>
+        <v>0.06</v>
       </c>
       <c r="G14" t="inlineStr"/>
     </row>
@@ -883,7 +883,7 @@
         </is>
       </c>
       <c r="F15" t="n">
-        <v>0.11</v>
+        <v>0.13</v>
       </c>
       <c r="G15" t="inlineStr"/>
     </row>
@@ -914,7 +914,7 @@
         </is>
       </c>
       <c r="F16" t="n">
-        <v>0.09</v>
+        <v>0.1</v>
       </c>
       <c r="G16" t="inlineStr"/>
     </row>
@@ -945,7 +945,7 @@
         </is>
       </c>
       <c r="F17" t="n">
-        <v>0.25</v>
+        <v>0.09</v>
       </c>
       <c r="G17" t="inlineStr"/>
     </row>
@@ -976,7 +976,7 @@
         </is>
       </c>
       <c r="F18" t="n">
-        <v>0.11</v>
+        <v>0.13</v>
       </c>
       <c r="G18" t="inlineStr"/>
     </row>
@@ -1007,7 +1007,7 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>0.12</v>
+        <v>0.06</v>
       </c>
       <c r="G19" t="inlineStr"/>
     </row>
@@ -1038,7 +1038,7 @@
         </is>
       </c>
       <c r="F20" t="n">
-        <v>0.15</v>
+        <v>0.14</v>
       </c>
       <c r="G20" t="inlineStr"/>
     </row>
@@ -1069,7 +1069,7 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.08</v>
       </c>
       <c r="G21" t="inlineStr"/>
     </row>
@@ -1100,7 +1100,7 @@
         </is>
       </c>
       <c r="F22" t="n">
-        <v>0.16</v>
+        <v>0.22</v>
       </c>
       <c r="G22" t="inlineStr"/>
     </row>
@@ -1162,7 +1162,7 @@
         </is>
       </c>
       <c r="F24" t="n">
-        <v>0.17</v>
+        <v>0.08</v>
       </c>
       <c r="G24" t="inlineStr"/>
     </row>
@@ -1193,7 +1193,7 @@
         </is>
       </c>
       <c r="F25" t="n">
-        <v>0.17</v>
+        <v>0.25</v>
       </c>
       <c r="G25" t="inlineStr"/>
     </row>
@@ -1224,7 +1224,7 @@
         </is>
       </c>
       <c r="F26" t="n">
-        <v>0.24</v>
+        <v>0.22</v>
       </c>
       <c r="G26" t="inlineStr"/>
     </row>
@@ -1255,7 +1255,7 @@
         </is>
       </c>
       <c r="F27" t="n">
-        <v>0.13</v>
+        <v>0.23</v>
       </c>
       <c r="G27" t="inlineStr"/>
     </row>
@@ -1286,7 +1286,7 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>0.08</v>
+        <v>0.15</v>
       </c>
       <c r="G28" t="inlineStr"/>
     </row>
@@ -1317,7 +1317,7 @@
         </is>
       </c>
       <c r="F29" t="n">
-        <v>0.23</v>
+        <v>0.18</v>
       </c>
       <c r="G29" t="inlineStr"/>
     </row>
@@ -1348,7 +1348,7 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>0.2</v>
+        <v>0.17</v>
       </c>
       <c r="G30" t="inlineStr"/>
     </row>
@@ -1379,7 +1379,7 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>0.16</v>
+        <v>0.21</v>
       </c>
       <c r="G31" t="inlineStr"/>
     </row>
@@ -1410,7 +1410,7 @@
         </is>
       </c>
       <c r="F32" t="n">
-        <v>0.14</v>
+        <v>0.1</v>
       </c>
       <c r="G32" t="inlineStr"/>
     </row>
@@ -1441,7 +1441,7 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>0.09</v>
+        <v>0.17</v>
       </c>
       <c r="G33" t="inlineStr"/>
     </row>
@@ -1472,7 +1472,7 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>0.14</v>
+        <v>0.05</v>
       </c>
       <c r="G34" t="inlineStr"/>
     </row>
@@ -1503,7 +1503,7 @@
         </is>
       </c>
       <c r="F35" t="n">
-        <v>0.19</v>
+        <v>0.14</v>
       </c>
       <c r="G35" t="inlineStr"/>
     </row>
@@ -1534,7 +1534,7 @@
         </is>
       </c>
       <c r="F36" t="n">
-        <v>0.22</v>
+        <v>0.21</v>
       </c>
       <c r="G36" t="inlineStr"/>
     </row>
@@ -1565,7 +1565,7 @@
         </is>
       </c>
       <c r="F37" t="n">
-        <v>0.22</v>
+        <v>0.19</v>
       </c>
       <c r="G37" t="inlineStr"/>
     </row>
@@ -1596,7 +1596,7 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>0.12</v>
+        <v>0.24</v>
       </c>
       <c r="G38" t="inlineStr"/>
     </row>
@@ -1627,7 +1627,7 @@
         </is>
       </c>
       <c r="F39" t="n">
-        <v>0.06</v>
+        <v>0.16</v>
       </c>
       <c r="G39" t="inlineStr"/>
     </row>
@@ -1658,7 +1658,7 @@
         </is>
       </c>
       <c r="F40" t="n">
-        <v>0.05</v>
+        <v>0.23</v>
       </c>
       <c r="G40" t="inlineStr"/>
     </row>
@@ -1689,7 +1689,7 @@
         </is>
       </c>
       <c r="F41" t="n">
-        <v>0.23</v>
+        <v>0.12</v>
       </c>
       <c r="G41" t="inlineStr"/>
     </row>
@@ -1720,7 +1720,7 @@
         </is>
       </c>
       <c r="F42" t="n">
-        <v>0.22</v>
+        <v>0.15</v>
       </c>
       <c r="G42" t="inlineStr"/>
     </row>
@@ -1751,7 +1751,7 @@
         </is>
       </c>
       <c r="F43" t="n">
-        <v>0.19</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="G43" t="inlineStr"/>
     </row>
@@ -1782,7 +1782,7 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>0.24</v>
+        <v>0.06</v>
       </c>
       <c r="G44" t="inlineStr"/>
     </row>
@@ -1813,7 +1813,7 @@
         </is>
       </c>
       <c r="F45" t="n">
-        <v>0.19</v>
+        <v>0.05</v>
       </c>
       <c r="G45" t="inlineStr"/>
     </row>
@@ -1844,7 +1844,7 @@
         </is>
       </c>
       <c r="F46" t="n">
-        <v>0.12</v>
+        <v>0.09</v>
       </c>
       <c r="G46" t="inlineStr"/>
     </row>
@@ -1875,7 +1875,7 @@
         </is>
       </c>
       <c r="F47" t="n">
-        <v>0.23</v>
+        <v>0.09</v>
       </c>
       <c r="G47" t="inlineStr"/>
     </row>
@@ -1906,7 +1906,7 @@
         </is>
       </c>
       <c r="F48" t="n">
-        <v>0.24</v>
+        <v>0.17</v>
       </c>
       <c r="G48" t="inlineStr"/>
     </row>
@@ -1937,7 +1937,7 @@
         </is>
       </c>
       <c r="F49" t="n">
-        <v>0.09</v>
+        <v>0.14</v>
       </c>
       <c r="G49" t="inlineStr"/>
     </row>
@@ -1968,7 +1968,7 @@
         </is>
       </c>
       <c r="F50" t="n">
-        <v>0.25</v>
+        <v>0.14</v>
       </c>
       <c r="G50" t="inlineStr"/>
     </row>
@@ -1999,7 +1999,7 @@
         </is>
       </c>
       <c r="F51" t="n">
-        <v>0.16</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="G51" t="inlineStr"/>
     </row>
@@ -2030,7 +2030,7 @@
         </is>
       </c>
       <c r="F52" t="n">
-        <v>0.22</v>
+        <v>0.06</v>
       </c>
       <c r="G52" t="inlineStr"/>
     </row>
@@ -2061,7 +2061,7 @@
         </is>
       </c>
       <c r="F53" t="n">
-        <v>0.1</v>
+        <v>0.19</v>
       </c>
       <c r="G53" t="inlineStr"/>
     </row>
@@ -2092,7 +2092,7 @@
         </is>
       </c>
       <c r="F54" t="n">
-        <v>0.09</v>
+        <v>0.19</v>
       </c>
       <c r="G54" t="inlineStr"/>
     </row>
@@ -2123,7 +2123,7 @@
         </is>
       </c>
       <c r="F55" t="n">
-        <v>0.21</v>
+        <v>0.12</v>
       </c>
       <c r="G55" t="inlineStr"/>
     </row>
@@ -2154,7 +2154,7 @@
         </is>
       </c>
       <c r="F56" t="n">
-        <v>0.23</v>
+        <v>0.21</v>
       </c>
       <c r="G56" t="inlineStr"/>
     </row>
@@ -2185,7 +2185,7 @@
         </is>
       </c>
       <c r="F57" t="n">
-        <v>0.24</v>
+        <v>0.15</v>
       </c>
       <c r="G57" t="inlineStr"/>
     </row>
@@ -2216,7 +2216,7 @@
         </is>
       </c>
       <c r="F58" t="n">
-        <v>0.12</v>
+        <v>0.18</v>
       </c>
       <c r="G58" t="inlineStr"/>
     </row>
@@ -2247,7 +2247,7 @@
         </is>
       </c>
       <c r="F59" t="n">
-        <v>0.14</v>
+        <v>0.19</v>
       </c>
       <c r="G59" t="inlineStr"/>
     </row>
@@ -2278,7 +2278,7 @@
         </is>
       </c>
       <c r="F60" t="n">
-        <v>0.19</v>
+        <v>0.15</v>
       </c>
       <c r="G60" t="inlineStr"/>
     </row>
@@ -2309,7 +2309,7 @@
         </is>
       </c>
       <c r="F61" t="n">
-        <v>0.06</v>
+        <v>0.18</v>
       </c>
       <c r="G61" t="inlineStr"/>
     </row>
@@ -2340,7 +2340,7 @@
         </is>
       </c>
       <c r="F62" t="n">
-        <v>0.11</v>
+        <v>0.18</v>
       </c>
       <c r="G62" t="inlineStr"/>
     </row>
@@ -2371,7 +2371,7 @@
         </is>
       </c>
       <c r="F63" t="n">
-        <v>0.08</v>
+        <v>0.17</v>
       </c>
       <c r="G63" t="inlineStr"/>
     </row>
@@ -2402,7 +2402,7 @@
         </is>
       </c>
       <c r="F64" t="n">
-        <v>0.24</v>
+        <v>0.22</v>
       </c>
       <c r="G64" t="inlineStr"/>
     </row>
@@ -2433,7 +2433,7 @@
         </is>
       </c>
       <c r="F65" t="n">
-        <v>0.17</v>
+        <v>0.13</v>
       </c>
       <c r="G65" t="inlineStr"/>
     </row>
@@ -2464,7 +2464,7 @@
         </is>
       </c>
       <c r="F66" t="n">
-        <v>0.18</v>
+        <v>0.1</v>
       </c>
       <c r="G66" t="inlineStr"/>
     </row>
@@ -2495,7 +2495,7 @@
         </is>
       </c>
       <c r="F67" t="n">
-        <v>0.1</v>
+        <v>0.16</v>
       </c>
       <c r="G67" t="inlineStr"/>
     </row>
@@ -2526,7 +2526,7 @@
         </is>
       </c>
       <c r="F68" t="n">
-        <v>0.21</v>
+        <v>0.11</v>
       </c>
       <c r="G68" t="inlineStr"/>
     </row>
@@ -2557,7 +2557,7 @@
         </is>
       </c>
       <c r="F69" t="n">
-        <v>0.11</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="G69" t="inlineStr"/>
     </row>
@@ -2588,7 +2588,7 @@
         </is>
       </c>
       <c r="F70" t="n">
-        <v>0.05</v>
+        <v>0.21</v>
       </c>
       <c r="G70" t="inlineStr"/>
     </row>
@@ -2619,7 +2619,7 @@
         </is>
       </c>
       <c r="F71" t="n">
-        <v>0.23</v>
+        <v>0.11</v>
       </c>
       <c r="G71" t="inlineStr"/>
     </row>
@@ -2650,7 +2650,7 @@
         </is>
       </c>
       <c r="F72" t="n">
-        <v>0.15</v>
+        <v>0.17</v>
       </c>
       <c r="G72" t="inlineStr"/>
     </row>
@@ -2712,7 +2712,7 @@
         </is>
       </c>
       <c r="F74" t="n">
-        <v>0.14</v>
+        <v>0.23</v>
       </c>
       <c r="G74" t="inlineStr"/>
     </row>
@@ -2743,7 +2743,7 @@
         </is>
       </c>
       <c r="F75" t="n">
-        <v>0.21</v>
+        <v>0.08</v>
       </c>
       <c r="G75" t="inlineStr"/>
     </row>
@@ -2774,7 +2774,7 @@
         </is>
       </c>
       <c r="F76" t="n">
-        <v>0.21</v>
+        <v>0.24</v>
       </c>
       <c r="G76" t="inlineStr"/>
     </row>
@@ -2805,7 +2805,7 @@
         </is>
       </c>
       <c r="F77" t="n">
-        <v>0.11</v>
+        <v>0.14</v>
       </c>
       <c r="G77" t="inlineStr"/>
     </row>
@@ -2836,7 +2836,7 @@
         </is>
       </c>
       <c r="F78" t="n">
-        <v>0.09</v>
+        <v>0.17</v>
       </c>
       <c r="G78" t="inlineStr"/>
     </row>
@@ -2867,7 +2867,7 @@
         </is>
       </c>
       <c r="F79" t="n">
-        <v>0.25</v>
+        <v>0.15</v>
       </c>
       <c r="G79" t="inlineStr"/>
     </row>
@@ -2898,7 +2898,7 @@
         </is>
       </c>
       <c r="F80" t="n">
-        <v>0.23</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="G80" t="inlineStr"/>
     </row>
@@ -2929,7 +2929,7 @@
         </is>
       </c>
       <c r="F81" t="n">
-        <v>0.15</v>
+        <v>0.09</v>
       </c>
       <c r="G81" t="inlineStr"/>
     </row>
@@ -2960,7 +2960,7 @@
         </is>
       </c>
       <c r="F82" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="G82" t="inlineStr"/>
     </row>
@@ -2991,7 +2991,7 @@
         </is>
       </c>
       <c r="F83" t="n">
-        <v>0.13</v>
+        <v>0.08</v>
       </c>
       <c r="G83" t="inlineStr"/>
     </row>
@@ -3022,7 +3022,7 @@
         </is>
       </c>
       <c r="F84" t="n">
-        <v>0.24</v>
+        <v>0.16</v>
       </c>
       <c r="G84" t="inlineStr"/>
     </row>
@@ -3053,7 +3053,7 @@
         </is>
       </c>
       <c r="F85" t="n">
-        <v>0.23</v>
+        <v>0.24</v>
       </c>
       <c r="G85" t="inlineStr"/>
     </row>
@@ -3084,7 +3084,7 @@
         </is>
       </c>
       <c r="F86" t="n">
-        <v>0.12</v>
+        <v>0.13</v>
       </c>
       <c r="G86" t="inlineStr"/>
     </row>
@@ -3115,7 +3115,7 @@
         </is>
       </c>
       <c r="F87" t="n">
-        <v>0.13</v>
+        <v>0.14</v>
       </c>
       <c r="G87" t="inlineStr"/>
     </row>
@@ -3146,7 +3146,7 @@
         </is>
       </c>
       <c r="F88" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.1</v>
       </c>
       <c r="G88" t="inlineStr"/>
     </row>
@@ -3177,7 +3177,7 @@
         </is>
       </c>
       <c r="F89" t="n">
-        <v>0.2</v>
+        <v>0.17</v>
       </c>
       <c r="G89" t="inlineStr"/>
     </row>
@@ -3208,7 +3208,7 @@
         </is>
       </c>
       <c r="F90" t="n">
-        <v>0.12</v>
+        <v>0.2</v>
       </c>
       <c r="G90" t="inlineStr"/>
     </row>
@@ -3239,7 +3239,7 @@
         </is>
       </c>
       <c r="F91" t="n">
-        <v>0.05</v>
+        <v>0.16</v>
       </c>
       <c r="G91" t="inlineStr"/>
     </row>
@@ -3270,7 +3270,7 @@
         </is>
       </c>
       <c r="F92" t="n">
-        <v>0.06</v>
+        <v>0.16</v>
       </c>
       <c r="G92" t="inlineStr"/>
     </row>
@@ -3301,7 +3301,7 @@
         </is>
       </c>
       <c r="F93" t="n">
-        <v>0.12</v>
+        <v>0.2</v>
       </c>
       <c r="G93" t="inlineStr"/>
     </row>
@@ -3332,7 +3332,7 @@
         </is>
       </c>
       <c r="F94" t="n">
-        <v>0.16</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="G94" t="inlineStr"/>
     </row>
@@ -3363,7 +3363,7 @@
         </is>
       </c>
       <c r="F95" t="n">
-        <v>0.24</v>
+        <v>0.18</v>
       </c>
       <c r="G95" t="inlineStr"/>
     </row>
@@ -3394,7 +3394,7 @@
         </is>
       </c>
       <c r="F96" t="n">
-        <v>0.05</v>
+        <v>0.2</v>
       </c>
       <c r="G96" t="inlineStr"/>
     </row>
@@ -3425,7 +3425,7 @@
         </is>
       </c>
       <c r="F97" t="n">
-        <v>0.24</v>
+        <v>0.05</v>
       </c>
       <c r="G97" t="inlineStr"/>
     </row>
@@ -3456,7 +3456,7 @@
         </is>
       </c>
       <c r="F98" t="n">
-        <v>0.18</v>
+        <v>0.1</v>
       </c>
       <c r="G98" t="inlineStr"/>
     </row>
@@ -3487,7 +3487,7 @@
         </is>
       </c>
       <c r="F99" t="n">
-        <v>0.21</v>
+        <v>0.16</v>
       </c>
       <c r="G99" t="inlineStr"/>
     </row>
@@ -3518,7 +3518,7 @@
         </is>
       </c>
       <c r="F100" t="n">
-        <v>0.17</v>
+        <v>0.15</v>
       </c>
       <c r="G100" t="inlineStr"/>
     </row>
@@ -3549,7 +3549,7 @@
         </is>
       </c>
       <c r="F101" t="n">
-        <v>0.12</v>
+        <v>0.08</v>
       </c>
       <c r="G101" t="inlineStr"/>
     </row>
@@ -3580,7 +3580,7 @@
         </is>
       </c>
       <c r="F102" t="n">
-        <v>0.19</v>
+        <v>0.11</v>
       </c>
       <c r="G102" t="inlineStr"/>
     </row>
@@ -3611,7 +3611,7 @@
         </is>
       </c>
       <c r="F103" t="n">
-        <v>0.22</v>
+        <v>0.19</v>
       </c>
       <c r="G103" t="inlineStr"/>
     </row>
@@ -3642,7 +3642,7 @@
         </is>
       </c>
       <c r="F104" t="n">
-        <v>0.17</v>
+        <v>0.21</v>
       </c>
       <c r="G104" t="inlineStr"/>
     </row>
@@ -3673,7 +3673,7 @@
         </is>
       </c>
       <c r="F105" t="n">
-        <v>0.16</v>
+        <v>0.19</v>
       </c>
       <c r="G105" t="inlineStr"/>
     </row>
@@ -3704,7 +3704,7 @@
         </is>
       </c>
       <c r="F106" t="n">
-        <v>0.17</v>
+        <v>0.11</v>
       </c>
       <c r="G106" t="inlineStr"/>
     </row>
@@ -3735,7 +3735,7 @@
         </is>
       </c>
       <c r="F107" t="n">
-        <v>0.09</v>
+        <v>0.16</v>
       </c>
       <c r="G107" t="inlineStr"/>
     </row>
@@ -3766,7 +3766,7 @@
         </is>
       </c>
       <c r="F108" t="n">
-        <v>0.15</v>
+        <v>0.14</v>
       </c>
       <c r="G108" t="inlineStr"/>
     </row>
@@ -3797,7 +3797,7 @@
         </is>
       </c>
       <c r="F109" t="n">
-        <v>0.11</v>
+        <v>0.24</v>
       </c>
       <c r="G109" t="inlineStr"/>
     </row>
@@ -3828,7 +3828,7 @@
         </is>
       </c>
       <c r="F110" t="n">
-        <v>0.11</v>
+        <v>0.08</v>
       </c>
       <c r="G110" t="inlineStr"/>
     </row>
@@ -3859,7 +3859,7 @@
         </is>
       </c>
       <c r="F111" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.21</v>
       </c>
       <c r="G111" t="inlineStr"/>
     </row>
@@ -3890,7 +3890,7 @@
         </is>
       </c>
       <c r="F112" t="n">
-        <v>0.13</v>
+        <v>0.25</v>
       </c>
       <c r="G112" t="inlineStr"/>
     </row>
@@ -3921,7 +3921,7 @@
         </is>
       </c>
       <c r="F113" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.22</v>
       </c>
       <c r="G113" t="inlineStr"/>
     </row>
@@ -3952,7 +3952,7 @@
         </is>
       </c>
       <c r="F114" t="n">
-        <v>0.23</v>
+        <v>0.12</v>
       </c>
       <c r="G114" t="inlineStr"/>
     </row>
@@ -4014,7 +4014,7 @@
         </is>
       </c>
       <c r="F116" t="n">
-        <v>0.24</v>
+        <v>0.06</v>
       </c>
       <c r="G116" t="inlineStr"/>
     </row>
@@ -4045,7 +4045,7 @@
         </is>
       </c>
       <c r="F117" t="n">
-        <v>0.15</v>
+        <v>0.11</v>
       </c>
       <c r="G117" t="inlineStr"/>
     </row>
@@ -4076,7 +4076,7 @@
         </is>
       </c>
       <c r="F118" t="n">
-        <v>0.23</v>
+        <v>0.16</v>
       </c>
       <c r="G118" t="inlineStr"/>
     </row>
@@ -4107,7 +4107,7 @@
         </is>
       </c>
       <c r="F119" t="n">
-        <v>0.12</v>
+        <v>0.05</v>
       </c>
       <c r="G119" t="inlineStr"/>
     </row>
@@ -4138,7 +4138,7 @@
         </is>
       </c>
       <c r="F120" t="n">
-        <v>0.11</v>
+        <v>0.08</v>
       </c>
       <c r="G120" t="inlineStr"/>
     </row>
@@ -4169,7 +4169,7 @@
         </is>
       </c>
       <c r="F121" t="n">
-        <v>0.2</v>
+        <v>0.12</v>
       </c>
       <c r="G121" t="inlineStr"/>
     </row>
@@ -4200,7 +4200,7 @@
         </is>
       </c>
       <c r="F122" t="n">
-        <v>0.18</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="G122" t="inlineStr"/>
     </row>
@@ -4231,7 +4231,7 @@
         </is>
       </c>
       <c r="F123" t="n">
-        <v>0.25</v>
+        <v>0.17</v>
       </c>
       <c r="G123" t="inlineStr"/>
     </row>
@@ -4262,7 +4262,7 @@
         </is>
       </c>
       <c r="F124" t="n">
-        <v>0.1</v>
+        <v>0.12</v>
       </c>
       <c r="G124" t="inlineStr"/>
     </row>
@@ -4293,7 +4293,7 @@
         </is>
       </c>
       <c r="F125" t="n">
-        <v>0.23</v>
+        <v>0.16</v>
       </c>
       <c r="G125" t="inlineStr"/>
     </row>
@@ -4324,7 +4324,7 @@
         </is>
       </c>
       <c r="F126" t="n">
-        <v>0.13</v>
+        <v>0.09</v>
       </c>
       <c r="G126" t="inlineStr"/>
     </row>
@@ -4355,7 +4355,7 @@
         </is>
       </c>
       <c r="F127" t="n">
-        <v>0.23</v>
+        <v>0.16</v>
       </c>
       <c r="G127" t="inlineStr"/>
     </row>
@@ -4386,7 +4386,7 @@
         </is>
       </c>
       <c r="F128" t="n">
-        <v>0.06</v>
+        <v>0.18</v>
       </c>
       <c r="G128" t="inlineStr"/>
     </row>
@@ -4417,7 +4417,7 @@
         </is>
       </c>
       <c r="F129" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="G129" t="inlineStr"/>
     </row>
@@ -4448,7 +4448,7 @@
         </is>
       </c>
       <c r="F130" t="n">
-        <v>0.13</v>
+        <v>0.23</v>
       </c>
       <c r="G130" t="inlineStr"/>
     </row>
@@ -4479,7 +4479,7 @@
         </is>
       </c>
       <c r="F131" t="n">
-        <v>0.11</v>
+        <v>0.08</v>
       </c>
       <c r="G131" t="inlineStr"/>
     </row>
@@ -4510,7 +4510,7 @@
         </is>
       </c>
       <c r="F132" t="n">
-        <v>0.2</v>
+        <v>0.16</v>
       </c>
       <c r="G132" t="inlineStr"/>
     </row>
@@ -4541,7 +4541,7 @@
         </is>
       </c>
       <c r="F133" t="n">
-        <v>0.13</v>
+        <v>0.22</v>
       </c>
       <c r="G133" t="inlineStr"/>
     </row>
@@ -4572,7 +4572,7 @@
         </is>
       </c>
       <c r="F134" t="n">
-        <v>0.14</v>
+        <v>0.19</v>
       </c>
       <c r="G134" t="inlineStr"/>
     </row>
@@ -4603,7 +4603,7 @@
         </is>
       </c>
       <c r="F135" t="n">
-        <v>0.18</v>
+        <v>0.19</v>
       </c>
       <c r="G135" t="inlineStr"/>
     </row>
@@ -4634,7 +4634,7 @@
         </is>
       </c>
       <c r="F136" t="n">
-        <v>0.1</v>
+        <v>0.17</v>
       </c>
       <c r="G136" t="inlineStr"/>
     </row>
@@ -4665,7 +4665,7 @@
         </is>
       </c>
       <c r="F137" t="n">
-        <v>0.12</v>
+        <v>0.08</v>
       </c>
       <c r="G137" t="inlineStr"/>
     </row>
@@ -4696,7 +4696,7 @@
         </is>
       </c>
       <c r="F138" t="n">
-        <v>0.13</v>
+        <v>0.17</v>
       </c>
       <c r="G138" t="inlineStr"/>
     </row>
@@ -4727,7 +4727,7 @@
         </is>
       </c>
       <c r="F139" t="n">
-        <v>0.21</v>
+        <v>0.05</v>
       </c>
       <c r="G139" t="inlineStr"/>
     </row>
@@ -4758,7 +4758,7 @@
         </is>
       </c>
       <c r="F140" t="n">
-        <v>0.06</v>
+        <v>0.25</v>
       </c>
       <c r="G140" t="inlineStr"/>
     </row>
@@ -4789,7 +4789,7 @@
         </is>
       </c>
       <c r="F141" t="n">
-        <v>0.23</v>
+        <v>0.05</v>
       </c>
       <c r="G141" t="inlineStr"/>
     </row>
@@ -4820,7 +4820,7 @@
         </is>
       </c>
       <c r="F142" t="n">
-        <v>0.16</v>
+        <v>0.1</v>
       </c>
       <c r="G142" t="inlineStr"/>
     </row>
@@ -4851,7 +4851,7 @@
         </is>
       </c>
       <c r="F143" t="n">
-        <v>0.21</v>
+        <v>0.18</v>
       </c>
       <c r="G143" t="inlineStr"/>
     </row>
@@ -4882,7 +4882,7 @@
         </is>
       </c>
       <c r="F144" t="n">
-        <v>0.13</v>
+        <v>0.19</v>
       </c>
       <c r="G144" t="inlineStr"/>
     </row>
@@ -4913,7 +4913,7 @@
         </is>
       </c>
       <c r="F145" t="n">
-        <v>0.21</v>
+        <v>0.09</v>
       </c>
       <c r="G145" t="inlineStr"/>
     </row>
@@ -4944,7 +4944,7 @@
         </is>
       </c>
       <c r="F146" t="n">
-        <v>0.06</v>
+        <v>0.14</v>
       </c>
       <c r="G146" t="inlineStr"/>
     </row>
@@ -4975,7 +4975,7 @@
         </is>
       </c>
       <c r="F147" t="n">
-        <v>0.22</v>
+        <v>0.12</v>
       </c>
       <c r="G147" t="inlineStr"/>
     </row>
@@ -5006,7 +5006,7 @@
         </is>
       </c>
       <c r="F148" t="n">
-        <v>0.05</v>
+        <v>0.21</v>
       </c>
       <c r="G148" t="inlineStr"/>
     </row>
@@ -5037,7 +5037,7 @@
         </is>
       </c>
       <c r="F149" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.11</v>
       </c>
       <c r="G149" t="inlineStr"/>
     </row>
@@ -5068,7 +5068,7 @@
         </is>
       </c>
       <c r="F150" t="n">
-        <v>0.1</v>
+        <v>0.18</v>
       </c>
       <c r="G150" t="inlineStr"/>
     </row>
@@ -5099,7 +5099,7 @@
         </is>
       </c>
       <c r="F151" t="n">
-        <v>0.13</v>
+        <v>0.1</v>
       </c>
       <c r="G151" t="inlineStr"/>
     </row>
@@ -5161,7 +5161,7 @@
         </is>
       </c>
       <c r="F153" t="n">
-        <v>0.14</v>
+        <v>0.22</v>
       </c>
       <c r="G153" t="inlineStr"/>
     </row>
@@ -5192,7 +5192,7 @@
         </is>
       </c>
       <c r="F154" t="n">
-        <v>0.23</v>
+        <v>0.24</v>
       </c>
       <c r="G154" t="inlineStr"/>
     </row>
@@ -5223,7 +5223,7 @@
         </is>
       </c>
       <c r="F155" t="n">
-        <v>0.09</v>
+        <v>0.21</v>
       </c>
       <c r="G155" t="inlineStr"/>
     </row>
@@ -5254,7 +5254,7 @@
         </is>
       </c>
       <c r="F156" t="n">
-        <v>0.1</v>
+        <v>0.12</v>
       </c>
       <c r="G156" t="inlineStr"/>
     </row>
@@ -5285,7 +5285,7 @@
         </is>
       </c>
       <c r="F157" t="n">
-        <v>0.16</v>
+        <v>0.06</v>
       </c>
       <c r="G157" t="inlineStr"/>
     </row>
@@ -5316,7 +5316,7 @@
         </is>
       </c>
       <c r="F158" t="n">
-        <v>0.09</v>
+        <v>0.06</v>
       </c>
       <c r="G158" t="inlineStr"/>
     </row>
@@ -5347,7 +5347,7 @@
         </is>
       </c>
       <c r="F159" t="n">
-        <v>0.17</v>
+        <v>0.09</v>
       </c>
       <c r="G159" t="inlineStr"/>
     </row>
@@ -5378,7 +5378,7 @@
         </is>
       </c>
       <c r="F160" t="n">
-        <v>0.15</v>
+        <v>0.19</v>
       </c>
       <c r="G160" t="inlineStr"/>
     </row>
@@ -5409,7 +5409,7 @@
         </is>
       </c>
       <c r="F161" t="n">
-        <v>0.22</v>
+        <v>0.06</v>
       </c>
       <c r="G161" t="inlineStr"/>
     </row>
@@ -5440,7 +5440,7 @@
         </is>
       </c>
       <c r="F162" t="n">
-        <v>0.2</v>
+        <v>0.17</v>
       </c>
       <c r="G162" t="inlineStr"/>
     </row>
@@ -5533,7 +5533,7 @@
         </is>
       </c>
       <c r="F165" t="n">
-        <v>0.16</v>
+        <v>0.09</v>
       </c>
       <c r="G165" t="inlineStr"/>
     </row>
@@ -5564,7 +5564,7 @@
         </is>
       </c>
       <c r="F166" t="n">
-        <v>0.24</v>
+        <v>0.21</v>
       </c>
       <c r="G166" t="inlineStr"/>
     </row>
@@ -5595,7 +5595,7 @@
         </is>
       </c>
       <c r="F167" t="n">
-        <v>0.16</v>
+        <v>0.24</v>
       </c>
       <c r="G167" t="inlineStr"/>
     </row>
@@ -5626,7 +5626,7 @@
         </is>
       </c>
       <c r="F168" t="n">
-        <v>0.19</v>
+        <v>0.18</v>
       </c>
       <c r="G168" t="inlineStr"/>
     </row>
@@ -5657,7 +5657,7 @@
         </is>
       </c>
       <c r="F169" t="n">
-        <v>0.23</v>
+        <v>0.21</v>
       </c>
       <c r="G169" t="inlineStr"/>
     </row>
@@ -5688,7 +5688,7 @@
         </is>
       </c>
       <c r="F170" t="n">
-        <v>0.15</v>
+        <v>0.08</v>
       </c>
       <c r="G170" t="inlineStr"/>
     </row>
@@ -5719,7 +5719,7 @@
         </is>
       </c>
       <c r="F171" t="n">
-        <v>0.08</v>
+        <v>0.06</v>
       </c>
       <c r="G171" t="inlineStr"/>
     </row>
@@ -5750,7 +5750,7 @@
         </is>
       </c>
       <c r="F172" t="n">
-        <v>0.11</v>
+        <v>0.06</v>
       </c>
       <c r="G172" t="inlineStr"/>
     </row>
@@ -5781,7 +5781,7 @@
         </is>
       </c>
       <c r="F173" t="n">
-        <v>0.09</v>
+        <v>0.18</v>
       </c>
       <c r="G173" t="inlineStr"/>
     </row>
@@ -5812,7 +5812,7 @@
         </is>
       </c>
       <c r="F174" t="n">
-        <v>0.15</v>
+        <v>0.16</v>
       </c>
       <c r="G174" t="inlineStr"/>
     </row>
@@ -5843,7 +5843,7 @@
         </is>
       </c>
       <c r="F175" t="n">
-        <v>0.09</v>
+        <v>0.15</v>
       </c>
       <c r="G175" t="inlineStr"/>
     </row>
@@ -5874,7 +5874,7 @@
         </is>
       </c>
       <c r="F176" t="n">
-        <v>0.16</v>
+        <v>0.25</v>
       </c>
       <c r="G176" t="inlineStr"/>
     </row>
@@ -5905,7 +5905,7 @@
         </is>
       </c>
       <c r="F177" t="n">
-        <v>0.14</v>
+        <v>0.11</v>
       </c>
       <c r="G177" t="inlineStr"/>
     </row>
@@ -5936,7 +5936,7 @@
         </is>
       </c>
       <c r="F178" t="n">
-        <v>0.09</v>
+        <v>0.24</v>
       </c>
       <c r="G178" t="inlineStr"/>
     </row>
@@ -5967,7 +5967,7 @@
         </is>
       </c>
       <c r="F179" t="n">
-        <v>0.16</v>
+        <v>0.13</v>
       </c>
       <c r="G179" t="inlineStr"/>
     </row>
@@ -5998,7 +5998,7 @@
         </is>
       </c>
       <c r="F180" t="n">
-        <v>0.06</v>
+        <v>0.1</v>
       </c>
       <c r="G180" t="inlineStr"/>
     </row>
@@ -6029,7 +6029,7 @@
         </is>
       </c>
       <c r="F181" t="n">
-        <v>0.18</v>
+        <v>0.05</v>
       </c>
       <c r="G181" t="inlineStr"/>
     </row>
@@ -6060,7 +6060,7 @@
         </is>
       </c>
       <c r="F182" t="n">
-        <v>0.06</v>
+        <v>0.16</v>
       </c>
       <c r="G182" t="inlineStr"/>
     </row>
@@ -6091,7 +6091,7 @@
         </is>
       </c>
       <c r="F183" t="n">
-        <v>0.12</v>
+        <v>0.18</v>
       </c>
       <c r="G183" t="inlineStr"/>
     </row>
@@ -6122,7 +6122,7 @@
         </is>
       </c>
       <c r="F184" t="n">
-        <v>0.22</v>
+        <v>0.17</v>
       </c>
       <c r="G184" t="inlineStr"/>
     </row>
@@ -6153,7 +6153,7 @@
         </is>
       </c>
       <c r="F185" t="n">
-        <v>0.08</v>
+        <v>0.19</v>
       </c>
       <c r="G185" t="inlineStr"/>
     </row>
@@ -6184,7 +6184,7 @@
         </is>
       </c>
       <c r="F186" t="n">
-        <v>0.15</v>
+        <v>0.22</v>
       </c>
       <c r="G186" t="inlineStr"/>
     </row>
@@ -6215,7 +6215,7 @@
         </is>
       </c>
       <c r="F187" t="n">
-        <v>0.11</v>
+        <v>0.06</v>
       </c>
       <c r="G187" t="inlineStr"/>
     </row>
@@ -6246,7 +6246,7 @@
         </is>
       </c>
       <c r="F188" t="n">
-        <v>0.14</v>
+        <v>0.08</v>
       </c>
       <c r="G188" t="inlineStr"/>
     </row>
@@ -6277,7 +6277,7 @@
         </is>
       </c>
       <c r="F189" t="n">
-        <v>0.08</v>
+        <v>0.16</v>
       </c>
       <c r="G189" t="inlineStr"/>
     </row>
@@ -6308,7 +6308,7 @@
         </is>
       </c>
       <c r="F190" t="n">
-        <v>0.21</v>
+        <v>0.14</v>
       </c>
       <c r="G190" t="inlineStr"/>
     </row>
@@ -6339,7 +6339,7 @@
         </is>
       </c>
       <c r="F191" t="n">
-        <v>0.2</v>
+        <v>0.24</v>
       </c>
       <c r="G191" t="inlineStr"/>
     </row>
@@ -6370,7 +6370,7 @@
         </is>
       </c>
       <c r="F192" t="n">
-        <v>0.06</v>
+        <v>0.23</v>
       </c>
       <c r="G192" t="inlineStr"/>
     </row>
@@ -6401,7 +6401,7 @@
         </is>
       </c>
       <c r="F193" t="n">
-        <v>0.23</v>
+        <v>0.19</v>
       </c>
       <c r="G193" t="inlineStr"/>
     </row>
@@ -6432,7 +6432,7 @@
         </is>
       </c>
       <c r="F194" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.14</v>
       </c>
       <c r="G194" t="inlineStr"/>
     </row>
@@ -6463,7 +6463,7 @@
         </is>
       </c>
       <c r="F195" t="n">
-        <v>0.21</v>
+        <v>0.1</v>
       </c>
       <c r="G195" t="inlineStr"/>
     </row>
@@ -6494,7 +6494,7 @@
         </is>
       </c>
       <c r="F196" t="n">
-        <v>0.22</v>
+        <v>0.21</v>
       </c>
       <c r="G196" t="inlineStr"/>
     </row>
@@ -6525,7 +6525,7 @@
         </is>
       </c>
       <c r="F197" t="n">
-        <v>0.22</v>
+        <v>0.12</v>
       </c>
       <c r="G197" t="inlineStr"/>
     </row>
@@ -6556,7 +6556,7 @@
         </is>
       </c>
       <c r="F198" t="n">
-        <v>0.08</v>
+        <v>0.11</v>
       </c>
       <c r="G198" t="inlineStr"/>
     </row>
@@ -6587,7 +6587,7 @@
         </is>
       </c>
       <c r="F199" t="n">
-        <v>0.08</v>
+        <v>0.12</v>
       </c>
       <c r="G199" t="inlineStr"/>
     </row>
@@ -6618,7 +6618,7 @@
         </is>
       </c>
       <c r="F200" t="n">
-        <v>0.22</v>
+        <v>0.08</v>
       </c>
       <c r="G200" t="inlineStr"/>
     </row>
@@ -6649,7 +6649,7 @@
         </is>
       </c>
       <c r="F201" t="n">
-        <v>0.2</v>
+        <v>0.23</v>
       </c>
       <c r="G201" t="inlineStr"/>
     </row>
@@ -6680,7 +6680,7 @@
         </is>
       </c>
       <c r="F202" t="n">
-        <v>0.24</v>
+        <v>0.18</v>
       </c>
       <c r="G202" t="inlineStr"/>
     </row>
@@ -6711,7 +6711,7 @@
         </is>
       </c>
       <c r="F203" t="n">
-        <v>0.18</v>
+        <v>0.15</v>
       </c>
       <c r="G203" t="inlineStr"/>
     </row>
@@ -6742,7 +6742,7 @@
         </is>
       </c>
       <c r="F204" t="n">
-        <v>0.15</v>
+        <v>0.22</v>
       </c>
       <c r="G204" t="inlineStr"/>
     </row>
@@ -6773,7 +6773,7 @@
         </is>
       </c>
       <c r="F205" t="n">
-        <v>0.12</v>
+        <v>0.22</v>
       </c>
       <c r="G205" t="inlineStr"/>
     </row>
@@ -6804,7 +6804,7 @@
         </is>
       </c>
       <c r="F206" t="n">
-        <v>0.13</v>
+        <v>0.11</v>
       </c>
       <c r="G206" t="inlineStr"/>
     </row>
@@ -6835,7 +6835,7 @@
         </is>
       </c>
       <c r="F207" t="n">
-        <v>0.05</v>
+        <v>0.11</v>
       </c>
       <c r="G207" t="inlineStr"/>
     </row>
@@ -6866,7 +6866,7 @@
         </is>
       </c>
       <c r="F208" t="n">
-        <v>0.05</v>
+        <v>0.2</v>
       </c>
       <c r="G208" t="inlineStr"/>
     </row>
@@ -6928,7 +6928,7 @@
         </is>
       </c>
       <c r="F210" t="n">
-        <v>0.15</v>
+        <v>0.23</v>
       </c>
       <c r="G210" t="inlineStr"/>
     </row>
@@ -6990,7 +6990,7 @@
         </is>
       </c>
       <c r="F212" t="n">
-        <v>0.15</v>
+        <v>0.18</v>
       </c>
       <c r="G212" t="inlineStr"/>
     </row>
@@ -7021,7 +7021,7 @@
         </is>
       </c>
       <c r="F213" t="n">
-        <v>0.08</v>
+        <v>0.1</v>
       </c>
       <c r="G213" t="inlineStr"/>
     </row>
@@ -7052,7 +7052,7 @@
         </is>
       </c>
       <c r="F214" t="n">
-        <v>0.13</v>
+        <v>0.16</v>
       </c>
       <c r="G214" t="inlineStr"/>
     </row>
@@ -7083,7 +7083,7 @@
         </is>
       </c>
       <c r="F215" t="n">
-        <v>0.16</v>
+        <v>0.06</v>
       </c>
       <c r="G215" t="inlineStr"/>
     </row>
@@ -7145,7 +7145,7 @@
         </is>
       </c>
       <c r="F217" t="n">
-        <v>0.17</v>
+        <v>0.13</v>
       </c>
       <c r="G217" t="inlineStr"/>
     </row>
@@ -7176,7 +7176,7 @@
         </is>
       </c>
       <c r="F218" t="n">
-        <v>0.21</v>
+        <v>0.19</v>
       </c>
       <c r="G218" t="inlineStr"/>
     </row>
@@ -7207,7 +7207,7 @@
         </is>
       </c>
       <c r="F219" t="n">
-        <v>0.11</v>
+        <v>0.16</v>
       </c>
       <c r="G219" t="inlineStr"/>
     </row>
@@ -7238,7 +7238,7 @@
         </is>
       </c>
       <c r="F220" t="n">
-        <v>0.17</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="G220" t="inlineStr"/>
     </row>
@@ -7269,7 +7269,7 @@
         </is>
       </c>
       <c r="F221" t="n">
-        <v>0.21</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="G221" t="inlineStr"/>
     </row>
@@ -7300,7 +7300,7 @@
         </is>
       </c>
       <c r="F222" t="n">
-        <v>0.2</v>
+        <v>0.13</v>
       </c>
       <c r="G222" t="inlineStr"/>
     </row>
@@ -7331,7 +7331,7 @@
         </is>
       </c>
       <c r="F223" t="n">
-        <v>0.22</v>
+        <v>0.2</v>
       </c>
       <c r="G223" t="inlineStr"/>
     </row>
@@ -7362,7 +7362,7 @@
         </is>
       </c>
       <c r="F224" t="n">
-        <v>0.12</v>
+        <v>0.11</v>
       </c>
       <c r="G224" t="inlineStr"/>
     </row>
@@ -7393,7 +7393,7 @@
         </is>
       </c>
       <c r="F225" t="n">
-        <v>0.12</v>
+        <v>0.13</v>
       </c>
       <c r="G225" t="inlineStr"/>
     </row>
@@ -7424,7 +7424,7 @@
         </is>
       </c>
       <c r="F226" t="n">
-        <v>0.19</v>
+        <v>0.09</v>
       </c>
       <c r="G226" t="inlineStr"/>
     </row>
@@ -7455,7 +7455,7 @@
         </is>
       </c>
       <c r="F227" t="n">
-        <v>0.16</v>
+        <v>0.06</v>
       </c>
       <c r="G227" t="inlineStr"/>
     </row>
@@ -7486,7 +7486,7 @@
         </is>
       </c>
       <c r="F228" t="n">
-        <v>0.19</v>
+        <v>0.18</v>
       </c>
       <c r="G228" t="inlineStr"/>
     </row>
@@ -7517,7 +7517,7 @@
         </is>
       </c>
       <c r="F229" t="n">
-        <v>0.11</v>
+        <v>0.16</v>
       </c>
       <c r="G229" t="inlineStr"/>
     </row>
@@ -7548,7 +7548,7 @@
         </is>
       </c>
       <c r="F230" t="n">
-        <v>0.23</v>
+        <v>0.24</v>
       </c>
       <c r="G230" t="inlineStr"/>
     </row>
@@ -7579,7 +7579,7 @@
         </is>
       </c>
       <c r="F231" t="n">
-        <v>0.2</v>
+        <v>0.22</v>
       </c>
       <c r="G231" t="inlineStr"/>
     </row>
@@ -7610,7 +7610,7 @@
         </is>
       </c>
       <c r="F232" t="n">
-        <v>0.12</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="G232" t="inlineStr"/>
     </row>
@@ -7641,7 +7641,7 @@
         </is>
       </c>
       <c r="F233" t="n">
-        <v>0.09</v>
+        <v>0.15</v>
       </c>
       <c r="G233" t="inlineStr"/>
     </row>
@@ -7672,7 +7672,7 @@
         </is>
       </c>
       <c r="F234" t="n">
-        <v>0.09</v>
+        <v>0.05</v>
       </c>
       <c r="G234" t="inlineStr"/>
     </row>
@@ -7703,7 +7703,7 @@
         </is>
       </c>
       <c r="F235" t="n">
-        <v>0.21</v>
+        <v>0.09</v>
       </c>
       <c r="G235" t="inlineStr"/>
     </row>
@@ -7734,7 +7734,7 @@
         </is>
       </c>
       <c r="F236" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.17</v>
       </c>
       <c r="G236" t="inlineStr"/>
     </row>
@@ -7765,7 +7765,7 @@
         </is>
       </c>
       <c r="F237" t="n">
-        <v>0.06</v>
+        <v>0.09</v>
       </c>
       <c r="G237" t="inlineStr"/>
     </row>
@@ -7796,7 +7796,7 @@
         </is>
       </c>
       <c r="F238" t="n">
-        <v>0.06</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="G238" t="inlineStr"/>
     </row>
@@ -7827,7 +7827,7 @@
         </is>
       </c>
       <c r="F239" t="n">
-        <v>0.13</v>
+        <v>0.09</v>
       </c>
       <c r="G239" t="inlineStr"/>
     </row>
@@ -7889,7 +7889,7 @@
         </is>
       </c>
       <c r="F241" t="n">
-        <v>0.17</v>
+        <v>0.1</v>
       </c>
       <c r="G241" t="inlineStr"/>
     </row>
@@ -7920,7 +7920,7 @@
         </is>
       </c>
       <c r="F242" t="n">
-        <v>0.05</v>
+        <v>0.12</v>
       </c>
       <c r="G242" t="inlineStr"/>
     </row>
@@ -7982,7 +7982,7 @@
         </is>
       </c>
       <c r="F244" t="n">
-        <v>0.05</v>
+        <v>0.2</v>
       </c>
       <c r="G244" t="inlineStr"/>
     </row>
@@ -8013,7 +8013,7 @@
         </is>
       </c>
       <c r="F245" t="n">
-        <v>0.06</v>
+        <v>0.1</v>
       </c>
       <c r="G245" t="inlineStr"/>
     </row>
@@ -8044,7 +8044,7 @@
         </is>
       </c>
       <c r="F246" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.06</v>
       </c>
       <c r="G246" t="inlineStr"/>
     </row>
@@ -8075,7 +8075,7 @@
         </is>
       </c>
       <c r="F247" t="n">
-        <v>0.16</v>
+        <v>0.08</v>
       </c>
       <c r="G247" t="inlineStr"/>
     </row>
@@ -8106,7 +8106,7 @@
         </is>
       </c>
       <c r="F248" t="n">
-        <v>0.16</v>
+        <v>0.1</v>
       </c>
       <c r="G248" t="inlineStr"/>
     </row>
@@ -8137,7 +8137,7 @@
         </is>
       </c>
       <c r="F249" t="n">
-        <v>0.15</v>
+        <v>0.22</v>
       </c>
       <c r="G249" t="inlineStr"/>
     </row>
@@ -8168,7 +8168,7 @@
         </is>
       </c>
       <c r="F250" t="n">
-        <v>0.05</v>
+        <v>0.2</v>
       </c>
       <c r="G250" t="inlineStr"/>
     </row>
@@ -8199,7 +8199,7 @@
         </is>
       </c>
       <c r="F251" t="n">
-        <v>0.09</v>
+        <v>0.1</v>
       </c>
       <c r="G251" t="inlineStr"/>
     </row>
@@ -8261,7 +8261,7 @@
         </is>
       </c>
       <c r="F253" t="n">
-        <v>0.06</v>
+        <v>0.13</v>
       </c>
       <c r="G253" t="inlineStr"/>
     </row>
@@ -8292,7 +8292,7 @@
         </is>
       </c>
       <c r="F254" t="n">
-        <v>0.19</v>
+        <v>0.11</v>
       </c>
       <c r="G254" t="inlineStr"/>
     </row>
@@ -8354,7 +8354,7 @@
         </is>
       </c>
       <c r="F256" t="n">
-        <v>0.09</v>
+        <v>0.23</v>
       </c>
       <c r="G256" t="inlineStr"/>
     </row>
@@ -8385,7 +8385,7 @@
         </is>
       </c>
       <c r="F257" t="n">
-        <v>0.13</v>
+        <v>0.12</v>
       </c>
       <c r="G257" t="inlineStr"/>
     </row>
@@ -8416,7 +8416,7 @@
         </is>
       </c>
       <c r="F258" t="n">
-        <v>0.2</v>
+        <v>0.09</v>
       </c>
       <c r="G258" t="inlineStr"/>
     </row>
@@ -8447,7 +8447,7 @@
         </is>
       </c>
       <c r="F259" t="n">
-        <v>0.08</v>
+        <v>0.15</v>
       </c>
       <c r="G259" t="inlineStr"/>
     </row>
@@ -8478,7 +8478,7 @@
         </is>
       </c>
       <c r="F260" t="n">
-        <v>0.16</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="G260" t="inlineStr"/>
     </row>
@@ -8509,7 +8509,7 @@
         </is>
       </c>
       <c r="F261" t="n">
-        <v>0.24</v>
+        <v>0.17</v>
       </c>
       <c r="G261" t="inlineStr"/>
     </row>
@@ -8540,7 +8540,7 @@
         </is>
       </c>
       <c r="F262" t="n">
-        <v>0.24</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="G262" t="inlineStr"/>
     </row>
@@ -8571,7 +8571,7 @@
         </is>
       </c>
       <c r="F263" t="n">
-        <v>0.23</v>
+        <v>0.06</v>
       </c>
       <c r="G263" t="inlineStr"/>
     </row>
@@ -8602,7 +8602,7 @@
         </is>
       </c>
       <c r="F264" t="n">
-        <v>0.12</v>
+        <v>0.1</v>
       </c>
       <c r="G264" t="inlineStr"/>
     </row>
@@ -8633,7 +8633,7 @@
         </is>
       </c>
       <c r="F265" t="n">
-        <v>0.25</v>
+        <v>0.16</v>
       </c>
       <c r="G265" t="inlineStr"/>
     </row>
@@ -8664,7 +8664,7 @@
         </is>
       </c>
       <c r="F266" t="n">
-        <v>0.14</v>
+        <v>0.17</v>
       </c>
       <c r="G266" t="inlineStr"/>
     </row>
@@ -8726,7 +8726,7 @@
         </is>
       </c>
       <c r="F268" t="n">
-        <v>0.24</v>
+        <v>0.15</v>
       </c>
       <c r="G268" t="inlineStr"/>
     </row>
@@ -8757,7 +8757,7 @@
         </is>
       </c>
       <c r="F269" t="n">
-        <v>0.2</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="G269" t="inlineStr"/>
     </row>
@@ -8788,7 +8788,7 @@
         </is>
       </c>
       <c r="F270" t="n">
-        <v>0.16</v>
+        <v>0.23</v>
       </c>
       <c r="G270" t="inlineStr"/>
     </row>
@@ -8819,7 +8819,7 @@
         </is>
       </c>
       <c r="F271" t="n">
-        <v>0.11</v>
+        <v>0.15</v>
       </c>
       <c r="G271" t="inlineStr"/>
     </row>
@@ -8850,7 +8850,7 @@
         </is>
       </c>
       <c r="F272" t="n">
-        <v>0.06</v>
+        <v>0.25</v>
       </c>
       <c r="G272" t="inlineStr"/>
     </row>
@@ -8881,7 +8881,7 @@
         </is>
       </c>
       <c r="F273" t="n">
-        <v>0.18</v>
+        <v>0.21</v>
       </c>
       <c r="G273" t="inlineStr"/>
     </row>
@@ -8912,7 +8912,7 @@
         </is>
       </c>
       <c r="F274" t="n">
-        <v>0.1</v>
+        <v>0.24</v>
       </c>
       <c r="G274" t="inlineStr"/>
     </row>
@@ -8943,7 +8943,7 @@
         </is>
       </c>
       <c r="F275" t="n">
-        <v>0.13</v>
+        <v>0.17</v>
       </c>
       <c r="G275" t="inlineStr"/>
     </row>
@@ -8974,7 +8974,7 @@
         </is>
       </c>
       <c r="F276" t="n">
-        <v>0.06</v>
+        <v>0.18</v>
       </c>
       <c r="G276" t="inlineStr"/>
     </row>
@@ -9005,7 +9005,7 @@
         </is>
       </c>
       <c r="F277" t="n">
-        <v>0.18</v>
+        <v>0.17</v>
       </c>
       <c r="G277" t="inlineStr"/>
     </row>
@@ -9067,7 +9067,7 @@
         </is>
       </c>
       <c r="F279" t="n">
-        <v>0.13</v>
+        <v>0.24</v>
       </c>
       <c r="G279" t="inlineStr"/>
     </row>
@@ -9098,7 +9098,7 @@
         </is>
       </c>
       <c r="F280" t="n">
-        <v>0.23</v>
+        <v>0.17</v>
       </c>
       <c r="G280" t="inlineStr"/>
     </row>
@@ -9129,7 +9129,7 @@
         </is>
       </c>
       <c r="F281" t="n">
-        <v>0.22</v>
+        <v>0.06</v>
       </c>
       <c r="G281" t="inlineStr"/>
     </row>
@@ -9160,7 +9160,7 @@
         </is>
       </c>
       <c r="F282" t="n">
-        <v>0.1</v>
+        <v>0.14</v>
       </c>
       <c r="G282" t="inlineStr"/>
     </row>
@@ -9222,7 +9222,7 @@
         </is>
       </c>
       <c r="F284" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.12</v>
       </c>
       <c r="G284" t="inlineStr"/>
     </row>
@@ -9253,7 +9253,7 @@
         </is>
       </c>
       <c r="F285" t="n">
-        <v>0.08</v>
+        <v>0.14</v>
       </c>
       <c r="G285" t="inlineStr"/>
     </row>
@@ -9284,7 +9284,7 @@
         </is>
       </c>
       <c r="F286" t="n">
-        <v>0.21</v>
+        <v>0.13</v>
       </c>
       <c r="G286" t="inlineStr"/>
     </row>
@@ -9315,7 +9315,7 @@
         </is>
       </c>
       <c r="F287" t="n">
-        <v>0.13</v>
+        <v>0.25</v>
       </c>
       <c r="G287" t="inlineStr"/>
     </row>
@@ -9346,7 +9346,7 @@
         </is>
       </c>
       <c r="F288" t="n">
-        <v>0.15</v>
+        <v>0.21</v>
       </c>
       <c r="G288" t="inlineStr"/>
     </row>
@@ -9377,7 +9377,7 @@
         </is>
       </c>
       <c r="F289" t="n">
-        <v>0.09</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="G289" t="inlineStr"/>
     </row>
@@ -9408,7 +9408,7 @@
         </is>
       </c>
       <c r="F290" t="n">
-        <v>0.16</v>
+        <v>0.14</v>
       </c>
       <c r="G290" t="inlineStr"/>
     </row>
@@ -9439,7 +9439,7 @@
         </is>
       </c>
       <c r="F291" t="n">
-        <v>0.22</v>
+        <v>0.14</v>
       </c>
       <c r="G291" t="inlineStr"/>
     </row>
@@ -9470,7 +9470,7 @@
         </is>
       </c>
       <c r="F292" t="n">
-        <v>0.11</v>
+        <v>0.09</v>
       </c>
       <c r="G292" t="inlineStr"/>
     </row>
@@ -9501,7 +9501,7 @@
         </is>
       </c>
       <c r="F293" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.2</v>
       </c>
       <c r="G293" t="inlineStr"/>
     </row>
@@ -9532,7 +9532,7 @@
         </is>
       </c>
       <c r="F294" t="n">
-        <v>0.15</v>
+        <v>0.12</v>
       </c>
       <c r="G294" t="inlineStr"/>
     </row>
@@ -9563,7 +9563,7 @@
         </is>
       </c>
       <c r="F295" t="n">
-        <v>0.16</v>
+        <v>0.12</v>
       </c>
       <c r="G295" t="inlineStr"/>
     </row>
@@ -9594,7 +9594,7 @@
         </is>
       </c>
       <c r="F296" t="n">
-        <v>0.15</v>
+        <v>0.11</v>
       </c>
       <c r="G296" t="inlineStr"/>
     </row>
@@ -9625,7 +9625,7 @@
         </is>
       </c>
       <c r="F297" t="n">
-        <v>0.19</v>
+        <v>0.21</v>
       </c>
       <c r="G297" t="inlineStr"/>
     </row>
@@ -9656,7 +9656,7 @@
         </is>
       </c>
       <c r="F298" t="n">
-        <v>0.13</v>
+        <v>0.05</v>
       </c>
       <c r="G298" t="inlineStr"/>
     </row>
@@ -9687,7 +9687,7 @@
         </is>
       </c>
       <c r="F299" t="n">
-        <v>0.24</v>
+        <v>0.12</v>
       </c>
       <c r="G299" t="inlineStr"/>
     </row>
@@ -9718,7 +9718,7 @@
         </is>
       </c>
       <c r="F300" t="n">
-        <v>0.17</v>
+        <v>0.11</v>
       </c>
       <c r="G300" t="inlineStr"/>
     </row>
@@ -9749,7 +9749,7 @@
         </is>
       </c>
       <c r="F301" t="n">
-        <v>0.11</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="G301" t="inlineStr"/>
     </row>
@@ -9780,7 +9780,7 @@
         </is>
       </c>
       <c r="F302" t="n">
-        <v>0.23</v>
+        <v>0.09</v>
       </c>
       <c r="G302" t="inlineStr"/>
     </row>
@@ -9811,7 +9811,7 @@
         </is>
       </c>
       <c r="F303" t="n">
-        <v>0.1</v>
+        <v>0.12</v>
       </c>
       <c r="G303" t="inlineStr"/>
     </row>
@@ -9842,7 +9842,7 @@
         </is>
       </c>
       <c r="F304" t="n">
-        <v>0.2</v>
+        <v>0.13</v>
       </c>
       <c r="G304" t="inlineStr"/>
     </row>
@@ -9873,7 +9873,7 @@
         </is>
       </c>
       <c r="F305" t="n">
-        <v>0.19</v>
+        <v>0.22</v>
       </c>
       <c r="G305" t="inlineStr"/>
     </row>
@@ -9904,7 +9904,7 @@
         </is>
       </c>
       <c r="F306" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.19</v>
       </c>
       <c r="G306" t="inlineStr"/>
     </row>
@@ -9935,7 +9935,7 @@
         </is>
       </c>
       <c r="F307" t="n">
-        <v>0.12</v>
+        <v>0.25</v>
       </c>
       <c r="G307" t="inlineStr"/>
     </row>
@@ -9966,7 +9966,7 @@
         </is>
       </c>
       <c r="F308" t="n">
-        <v>0.25</v>
+        <v>0.11</v>
       </c>
       <c r="G308" t="inlineStr"/>
     </row>
@@ -9997,7 +9997,7 @@
         </is>
       </c>
       <c r="F309" t="n">
-        <v>0.12</v>
+        <v>0.1</v>
       </c>
       <c r="G309" t="inlineStr"/>
     </row>
@@ -10028,7 +10028,7 @@
         </is>
       </c>
       <c r="F310" t="n">
-        <v>0.21</v>
+        <v>0.17</v>
       </c>
       <c r="G310" t="inlineStr"/>
     </row>
@@ -10059,7 +10059,7 @@
         </is>
       </c>
       <c r="F311" t="n">
-        <v>0.16</v>
+        <v>0.05</v>
       </c>
       <c r="G311" t="inlineStr"/>
     </row>
@@ -10090,7 +10090,7 @@
         </is>
       </c>
       <c r="F312" t="n">
-        <v>0.11</v>
+        <v>0.18</v>
       </c>
       <c r="G312" t="inlineStr"/>
     </row>
@@ -10121,7 +10121,7 @@
         </is>
       </c>
       <c r="F313" t="n">
-        <v>0.21</v>
+        <v>0.19</v>
       </c>
       <c r="G313" t="inlineStr"/>
     </row>
@@ -10152,7 +10152,7 @@
         </is>
       </c>
       <c r="F314" t="n">
-        <v>0.06</v>
+        <v>0.17</v>
       </c>
       <c r="G314" t="inlineStr"/>
     </row>
@@ -10183,7 +10183,7 @@
         </is>
       </c>
       <c r="F315" t="n">
-        <v>0.12</v>
+        <v>0.19</v>
       </c>
       <c r="G315" t="inlineStr"/>
     </row>
@@ -10214,7 +10214,7 @@
         </is>
       </c>
       <c r="F316" t="n">
-        <v>0.1</v>
+        <v>0.22</v>
       </c>
       <c r="G316" t="inlineStr"/>
     </row>
@@ -10245,7 +10245,7 @@
         </is>
       </c>
       <c r="F317" t="n">
-        <v>0.23</v>
+        <v>0.13</v>
       </c>
       <c r="G317" t="inlineStr"/>
     </row>
@@ -10276,7 +10276,7 @@
         </is>
       </c>
       <c r="F318" t="n">
-        <v>0.24</v>
+        <v>0.15</v>
       </c>
       <c r="G318" t="inlineStr"/>
     </row>
@@ -10307,7 +10307,7 @@
         </is>
       </c>
       <c r="F319" t="n">
-        <v>0.08</v>
+        <v>0.25</v>
       </c>
       <c r="G319" t="inlineStr"/>
     </row>
@@ -10338,7 +10338,7 @@
         </is>
       </c>
       <c r="F320" t="n">
-        <v>0.09</v>
+        <v>0.12</v>
       </c>
       <c r="G320" t="inlineStr"/>
     </row>
@@ -10369,7 +10369,7 @@
         </is>
       </c>
       <c r="F321" t="n">
-        <v>0.05</v>
+        <v>0.15</v>
       </c>
       <c r="G321" t="inlineStr"/>
     </row>
@@ -10431,7 +10431,7 @@
         </is>
       </c>
       <c r="F323" t="n">
-        <v>0.12</v>
+        <v>0.19</v>
       </c>
       <c r="G323" t="inlineStr"/>
     </row>
@@ -10462,7 +10462,7 @@
         </is>
       </c>
       <c r="F324" t="n">
-        <v>0.14</v>
+        <v>0.19</v>
       </c>
       <c r="G324" t="inlineStr"/>
     </row>
@@ -10524,7 +10524,7 @@
         </is>
       </c>
       <c r="F326" t="n">
-        <v>0.15</v>
+        <v>0.22</v>
       </c>
       <c r="G326" t="inlineStr"/>
     </row>
@@ -10555,7 +10555,7 @@
         </is>
       </c>
       <c r="F327" t="n">
-        <v>0.06</v>
+        <v>0.08</v>
       </c>
       <c r="G327" t="inlineStr"/>
     </row>
@@ -10586,7 +10586,7 @@
         </is>
       </c>
       <c r="F328" t="n">
-        <v>0.2</v>
+        <v>0.13</v>
       </c>
       <c r="G328" t="inlineStr"/>
     </row>
@@ -10617,7 +10617,7 @@
         </is>
       </c>
       <c r="F329" t="n">
-        <v>0.13</v>
+        <v>0.06</v>
       </c>
       <c r="G329" t="inlineStr"/>
     </row>
@@ -10648,7 +10648,7 @@
         </is>
       </c>
       <c r="F330" t="n">
-        <v>0.25</v>
+        <v>0.2</v>
       </c>
       <c r="G330" t="inlineStr"/>
     </row>
@@ -10679,7 +10679,7 @@
         </is>
       </c>
       <c r="F331" t="n">
-        <v>0.24</v>
+        <v>0.22</v>
       </c>
       <c r="G331" t="inlineStr"/>
     </row>
@@ -10710,7 +10710,7 @@
         </is>
       </c>
       <c r="F332" t="n">
-        <v>0.23</v>
+        <v>0.18</v>
       </c>
       <c r="G332" t="inlineStr"/>
     </row>
@@ -10741,7 +10741,7 @@
         </is>
       </c>
       <c r="F333" t="n">
-        <v>0.14</v>
+        <v>0.13</v>
       </c>
       <c r="G333" t="inlineStr"/>
     </row>
@@ -10772,7 +10772,7 @@
         </is>
       </c>
       <c r="F334" t="n">
-        <v>0.21</v>
+        <v>0.1</v>
       </c>
       <c r="G334" t="inlineStr"/>
     </row>
@@ -10803,7 +10803,7 @@
         </is>
       </c>
       <c r="F335" t="n">
-        <v>0.06</v>
+        <v>0.24</v>
       </c>
       <c r="G335" t="inlineStr"/>
     </row>
@@ -10834,7 +10834,7 @@
         </is>
       </c>
       <c r="F336" t="n">
-        <v>0.16</v>
+        <v>0.1</v>
       </c>
       <c r="G336" t="inlineStr"/>
     </row>
@@ -10865,7 +10865,7 @@
         </is>
       </c>
       <c r="F337" t="n">
-        <v>0.25</v>
+        <v>0.08</v>
       </c>
       <c r="G337" t="inlineStr"/>
     </row>
@@ -10896,7 +10896,7 @@
         </is>
       </c>
       <c r="F338" t="n">
-        <v>0.09</v>
+        <v>0.08</v>
       </c>
       <c r="G338" t="inlineStr"/>
     </row>
@@ -10927,7 +10927,7 @@
         </is>
       </c>
       <c r="F339" t="n">
-        <v>0.1</v>
+        <v>0.11</v>
       </c>
       <c r="G339" t="inlineStr"/>
     </row>
@@ -10958,7 +10958,7 @@
         </is>
       </c>
       <c r="F340" t="n">
-        <v>0.19</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="G340" t="inlineStr"/>
     </row>
@@ -10989,7 +10989,7 @@
         </is>
       </c>
       <c r="F341" t="n">
-        <v>0.23</v>
+        <v>0.24</v>
       </c>
       <c r="G341" t="inlineStr"/>
     </row>
@@ -11020,7 +11020,7 @@
         </is>
       </c>
       <c r="F342" t="n">
-        <v>0.13</v>
+        <v>0.21</v>
       </c>
       <c r="G342" t="inlineStr"/>
     </row>
@@ -11051,7 +11051,7 @@
         </is>
       </c>
       <c r="F343" t="n">
-        <v>0.2</v>
+        <v>0.25</v>
       </c>
       <c r="G343" t="inlineStr"/>
     </row>
@@ -11082,7 +11082,7 @@
         </is>
       </c>
       <c r="F344" t="n">
-        <v>0.11</v>
+        <v>0.18</v>
       </c>
       <c r="G344" t="inlineStr"/>
     </row>
@@ -11113,7 +11113,7 @@
         </is>
       </c>
       <c r="F345" t="n">
-        <v>0.24</v>
+        <v>0.06</v>
       </c>
       <c r="G345" t="inlineStr"/>
     </row>
@@ -11144,7 +11144,7 @@
         </is>
       </c>
       <c r="F346" t="n">
-        <v>0.1</v>
+        <v>0.24</v>
       </c>
       <c r="G346" t="inlineStr"/>
     </row>
@@ -11175,7 +11175,7 @@
         </is>
       </c>
       <c r="F347" t="n">
-        <v>0.06</v>
+        <v>0.1</v>
       </c>
       <c r="G347" t="inlineStr"/>
     </row>
@@ -11206,7 +11206,7 @@
         </is>
       </c>
       <c r="F348" t="n">
-        <v>0.1</v>
+        <v>0.12</v>
       </c>
       <c r="G348" t="inlineStr"/>
     </row>
@@ -11237,7 +11237,7 @@
         </is>
       </c>
       <c r="F349" t="n">
-        <v>0.19</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="G349" t="inlineStr"/>
     </row>
@@ -11268,7 +11268,7 @@
         </is>
       </c>
       <c r="F350" t="n">
-        <v>0.12</v>
+        <v>0.09</v>
       </c>
       <c r="G350" t="inlineStr"/>
     </row>
@@ -11299,7 +11299,7 @@
         </is>
       </c>
       <c r="F351" t="n">
-        <v>0.13</v>
+        <v>0.21</v>
       </c>
       <c r="G351" t="inlineStr"/>
     </row>
@@ -11330,7 +11330,7 @@
         </is>
       </c>
       <c r="F352" t="n">
-        <v>0.21</v>
+        <v>0.23</v>
       </c>
       <c r="G352" t="inlineStr"/>
     </row>
@@ -11361,7 +11361,7 @@
         </is>
       </c>
       <c r="F353" t="n">
-        <v>0.12</v>
+        <v>0.18</v>
       </c>
       <c r="G353" t="inlineStr"/>
     </row>
@@ -11392,7 +11392,7 @@
         </is>
       </c>
       <c r="F354" t="n">
-        <v>0.14</v>
+        <v>0.18</v>
       </c>
       <c r="G354" t="inlineStr"/>
     </row>
@@ -11423,7 +11423,7 @@
         </is>
       </c>
       <c r="F355" t="n">
-        <v>0.09</v>
+        <v>0.13</v>
       </c>
       <c r="G355" t="inlineStr"/>
     </row>
@@ -11454,7 +11454,7 @@
         </is>
       </c>
       <c r="F356" t="n">
-        <v>0.15</v>
+        <v>0.16</v>
       </c>
       <c r="G356" t="inlineStr"/>
     </row>
@@ -11485,7 +11485,7 @@
         </is>
       </c>
       <c r="F357" t="n">
-        <v>0.13</v>
+        <v>0.08</v>
       </c>
       <c r="G357" t="inlineStr"/>
     </row>
@@ -11516,7 +11516,7 @@
         </is>
       </c>
       <c r="F358" t="n">
-        <v>0.06</v>
+        <v>0.12</v>
       </c>
       <c r="G358" t="inlineStr"/>
     </row>
@@ -11547,7 +11547,7 @@
         </is>
       </c>
       <c r="F359" t="n">
-        <v>0.18</v>
+        <v>0.24</v>
       </c>
       <c r="G359" t="inlineStr"/>
     </row>
@@ -11578,7 +11578,7 @@
         </is>
       </c>
       <c r="F360" t="n">
-        <v>0.19</v>
+        <v>0.24</v>
       </c>
       <c r="G360" t="inlineStr"/>
     </row>
@@ -11609,7 +11609,7 @@
         </is>
       </c>
       <c r="F361" t="n">
-        <v>0.17</v>
+        <v>0.15</v>
       </c>
       <c r="G361" t="inlineStr"/>
     </row>
@@ -11640,7 +11640,7 @@
         </is>
       </c>
       <c r="F362" t="n">
-        <v>0.23</v>
+        <v>0.2</v>
       </c>
       <c r="G362" t="inlineStr"/>
     </row>
@@ -11671,7 +11671,7 @@
         </is>
       </c>
       <c r="F363" t="n">
-        <v>0.23</v>
+        <v>0.17</v>
       </c>
       <c r="G363" t="inlineStr"/>
     </row>
@@ -11702,7 +11702,7 @@
         </is>
       </c>
       <c r="F364" t="n">
-        <v>0.22</v>
+        <v>0.17</v>
       </c>
       <c r="G364" t="inlineStr"/>
     </row>
@@ -11733,7 +11733,7 @@
         </is>
       </c>
       <c r="F365" t="n">
-        <v>0.09</v>
+        <v>0.16</v>
       </c>
       <c r="G365" t="inlineStr"/>
     </row>
@@ -11795,7 +11795,7 @@
         </is>
       </c>
       <c r="F367" t="n">
-        <v>0.13</v>
+        <v>0.12</v>
       </c>
       <c r="G367" t="inlineStr"/>
     </row>
@@ -11826,7 +11826,7 @@
         </is>
       </c>
       <c r="F368" t="n">
-        <v>0.2</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="G368" t="inlineStr"/>
     </row>
@@ -11857,7 +11857,7 @@
         </is>
       </c>
       <c r="F369" t="n">
-        <v>0.18</v>
+        <v>0.16</v>
       </c>
       <c r="G369" t="inlineStr"/>
     </row>
@@ -11888,7 +11888,7 @@
         </is>
       </c>
       <c r="F370" t="n">
-        <v>0.25</v>
+        <v>0.14</v>
       </c>
       <c r="G370" t="inlineStr"/>
     </row>
@@ -11950,7 +11950,7 @@
         </is>
       </c>
       <c r="F372" t="n">
-        <v>0.16</v>
+        <v>0.14</v>
       </c>
       <c r="G372" t="inlineStr"/>
     </row>
@@ -11981,7 +11981,7 @@
         </is>
       </c>
       <c r="F373" t="n">
-        <v>0.24</v>
+        <v>0.1</v>
       </c>
       <c r="G373" t="inlineStr"/>
     </row>
@@ -12012,7 +12012,7 @@
         </is>
       </c>
       <c r="F374" t="n">
-        <v>0.06</v>
+        <v>0.12</v>
       </c>
       <c r="G374" t="inlineStr"/>
     </row>
@@ -12043,7 +12043,7 @@
         </is>
       </c>
       <c r="F375" t="n">
-        <v>0.1</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="G375" t="inlineStr"/>
     </row>
@@ -12074,7 +12074,7 @@
         </is>
       </c>
       <c r="F376" t="n">
-        <v>0.18</v>
+        <v>0.17</v>
       </c>
       <c r="G376" t="inlineStr"/>
     </row>
@@ -12105,7 +12105,7 @@
         </is>
       </c>
       <c r="F377" t="n">
-        <v>0.23</v>
+        <v>0.18</v>
       </c>
       <c r="G377" t="inlineStr"/>
     </row>
@@ -12136,7 +12136,7 @@
         </is>
       </c>
       <c r="F378" t="n">
-        <v>0.23</v>
+        <v>0.14</v>
       </c>
       <c r="G378" t="inlineStr"/>
     </row>
@@ -12167,7 +12167,7 @@
         </is>
       </c>
       <c r="F379" t="n">
-        <v>0.18</v>
+        <v>0.05</v>
       </c>
       <c r="G379" t="inlineStr"/>
     </row>
@@ -12198,7 +12198,7 @@
         </is>
       </c>
       <c r="F380" t="n">
-        <v>0.16</v>
+        <v>0.23</v>
       </c>
       <c r="G380" t="inlineStr"/>
     </row>
@@ -12229,7 +12229,7 @@
         </is>
       </c>
       <c r="F381" t="n">
-        <v>0.17</v>
+        <v>0.12</v>
       </c>
       <c r="G381" t="inlineStr"/>
     </row>
@@ -12260,7 +12260,7 @@
         </is>
       </c>
       <c r="F382" t="n">
-        <v>0.21</v>
+        <v>0.24</v>
       </c>
       <c r="G382" t="inlineStr"/>
     </row>
@@ -12291,7 +12291,7 @@
         </is>
       </c>
       <c r="F383" t="n">
-        <v>0.18</v>
+        <v>0.17</v>
       </c>
       <c r="G383" t="inlineStr"/>
     </row>
@@ -12322,7 +12322,7 @@
         </is>
       </c>
       <c r="F384" t="n">
-        <v>0.15</v>
+        <v>0.16</v>
       </c>
       <c r="G384" t="inlineStr"/>
     </row>
@@ -12353,7 +12353,7 @@
         </is>
       </c>
       <c r="F385" t="n">
-        <v>0.15</v>
+        <v>0.17</v>
       </c>
       <c r="G385" t="inlineStr"/>
     </row>
@@ -12384,7 +12384,7 @@
         </is>
       </c>
       <c r="F386" t="n">
-        <v>0.12</v>
+        <v>0.17</v>
       </c>
       <c r="G386" t="inlineStr"/>
     </row>
@@ -12415,7 +12415,7 @@
         </is>
       </c>
       <c r="F387" t="n">
-        <v>0.06</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="G387" t="inlineStr"/>
     </row>
@@ -12446,7 +12446,7 @@
         </is>
       </c>
       <c r="F388" t="n">
-        <v>0.16</v>
+        <v>0.19</v>
       </c>
       <c r="G388" t="inlineStr"/>
     </row>
@@ -12477,7 +12477,7 @@
         </is>
       </c>
       <c r="F389" t="n">
-        <v>0.24</v>
+        <v>0.22</v>
       </c>
       <c r="G389" t="inlineStr"/>
     </row>
@@ -12508,7 +12508,7 @@
         </is>
       </c>
       <c r="F390" t="n">
-        <v>0.22</v>
+        <v>0.11</v>
       </c>
       <c r="G390" t="inlineStr"/>
     </row>
@@ -12539,7 +12539,7 @@
         </is>
       </c>
       <c r="F391" t="n">
-        <v>0.19</v>
+        <v>0.24</v>
       </c>
       <c r="G391" t="inlineStr"/>
     </row>
@@ -12570,7 +12570,7 @@
         </is>
       </c>
       <c r="F392" t="n">
-        <v>0.18</v>
+        <v>0.21</v>
       </c>
       <c r="G392" t="inlineStr"/>
     </row>
@@ -12601,7 +12601,7 @@
         </is>
       </c>
       <c r="F393" t="n">
-        <v>0.24</v>
+        <v>0.17</v>
       </c>
       <c r="G393" t="inlineStr"/>
     </row>
@@ -12632,7 +12632,7 @@
         </is>
       </c>
       <c r="F394" t="n">
-        <v>0.17</v>
+        <v>0.09</v>
       </c>
       <c r="G394" t="inlineStr"/>
     </row>
@@ -12663,7 +12663,7 @@
         </is>
       </c>
       <c r="F395" t="n">
-        <v>0.14</v>
+        <v>0.2</v>
       </c>
       <c r="G395" t="inlineStr"/>
     </row>
@@ -12694,7 +12694,7 @@
         </is>
       </c>
       <c r="F396" t="n">
-        <v>0.14</v>
+        <v>0.23</v>
       </c>
       <c r="G396" t="inlineStr"/>
     </row>
@@ -12725,7 +12725,7 @@
         </is>
       </c>
       <c r="F397" t="n">
-        <v>0.15</v>
+        <v>0.2</v>
       </c>
       <c r="G397" t="inlineStr"/>
     </row>
@@ -12756,7 +12756,7 @@
         </is>
       </c>
       <c r="F398" t="n">
-        <v>0.17</v>
+        <v>0.05</v>
       </c>
       <c r="G398" t="inlineStr"/>
     </row>
@@ -12818,7 +12818,7 @@
         </is>
       </c>
       <c r="F400" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.14</v>
       </c>
       <c r="G400" t="inlineStr"/>
     </row>
@@ -12849,7 +12849,7 @@
         </is>
       </c>
       <c r="F401" t="n">
-        <v>0.06</v>
+        <v>0.15</v>
       </c>
       <c r="G401" t="inlineStr"/>
     </row>
@@ -12880,7 +12880,7 @@
         </is>
       </c>
       <c r="F402" t="n">
-        <v>0.1</v>
+        <v>0.15</v>
       </c>
       <c r="G402" t="inlineStr"/>
     </row>
@@ -12911,7 +12911,7 @@
         </is>
       </c>
       <c r="F403" t="n">
-        <v>0.19</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="G403" t="inlineStr"/>
     </row>
@@ -12942,7 +12942,7 @@
         </is>
       </c>
       <c r="F404" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="G404" t="inlineStr"/>
     </row>
@@ -12973,7 +12973,7 @@
         </is>
       </c>
       <c r="F405" t="n">
-        <v>0.23</v>
+        <v>0.24</v>
       </c>
       <c r="G405" t="inlineStr"/>
     </row>
@@ -13004,7 +13004,7 @@
         </is>
       </c>
       <c r="F406" t="n">
-        <v>0.23</v>
+        <v>0.17</v>
       </c>
       <c r="G406" t="inlineStr"/>
     </row>
@@ -13035,7 +13035,7 @@
         </is>
       </c>
       <c r="F407" t="n">
-        <v>0.11</v>
+        <v>0.09</v>
       </c>
       <c r="G407" t="inlineStr"/>
     </row>
@@ -13097,7 +13097,7 @@
         </is>
       </c>
       <c r="F409" t="n">
-        <v>0.14</v>
+        <v>0.23</v>
       </c>
       <c r="G409" t="inlineStr"/>
     </row>
@@ -13128,7 +13128,7 @@
         </is>
       </c>
       <c r="F410" t="n">
-        <v>0.19</v>
+        <v>0.15</v>
       </c>
       <c r="G410" t="inlineStr"/>
     </row>
@@ -13159,7 +13159,7 @@
         </is>
       </c>
       <c r="F411" t="n">
-        <v>0.12</v>
+        <v>0.13</v>
       </c>
       <c r="G411" t="inlineStr"/>
     </row>
@@ -13190,7 +13190,7 @@
         </is>
       </c>
       <c r="F412" t="n">
-        <v>0.08</v>
+        <v>0.12</v>
       </c>
       <c r="G412" t="inlineStr"/>
     </row>
@@ -13221,7 +13221,7 @@
         </is>
       </c>
       <c r="F413" t="n">
-        <v>0.18</v>
+        <v>0.23</v>
       </c>
       <c r="G413" t="inlineStr"/>
     </row>
@@ -13252,7 +13252,7 @@
         </is>
       </c>
       <c r="F414" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="G414" t="inlineStr"/>
     </row>
@@ -13283,7 +13283,7 @@
         </is>
       </c>
       <c r="F415" t="n">
-        <v>0.24</v>
+        <v>0.1</v>
       </c>
       <c r="G415" t="inlineStr"/>
     </row>
@@ -13314,7 +13314,7 @@
         </is>
       </c>
       <c r="F416" t="n">
-        <v>0.13</v>
+        <v>0.09</v>
       </c>
       <c r="G416" t="inlineStr"/>
     </row>
@@ -13345,7 +13345,7 @@
         </is>
       </c>
       <c r="F417" t="n">
-        <v>0.11</v>
+        <v>0.06</v>
       </c>
       <c r="G417" t="inlineStr"/>
     </row>
@@ -13376,7 +13376,7 @@
         </is>
       </c>
       <c r="F418" t="n">
-        <v>0.24</v>
+        <v>0.13</v>
       </c>
       <c r="G418" t="inlineStr"/>
     </row>
@@ -13407,7 +13407,7 @@
         </is>
       </c>
       <c r="F419" t="n">
-        <v>0.14</v>
+        <v>0.21</v>
       </c>
       <c r="G419" t="inlineStr"/>
     </row>
@@ -13438,7 +13438,7 @@
         </is>
       </c>
       <c r="F420" t="n">
-        <v>0.11</v>
+        <v>0.2</v>
       </c>
       <c r="G420" t="inlineStr"/>
     </row>
@@ -13469,7 +13469,7 @@
         </is>
       </c>
       <c r="F421" t="n">
-        <v>0.05</v>
+        <v>0.17</v>
       </c>
       <c r="G421" t="inlineStr"/>
     </row>
@@ -13500,7 +13500,7 @@
         </is>
       </c>
       <c r="F422" t="n">
-        <v>0.11</v>
+        <v>0.06</v>
       </c>
       <c r="G422" t="inlineStr"/>
     </row>
@@ -13531,7 +13531,7 @@
         </is>
       </c>
       <c r="F423" t="n">
-        <v>0.23</v>
+        <v>0.06</v>
       </c>
       <c r="G423" t="inlineStr"/>
     </row>
@@ -13562,7 +13562,7 @@
         </is>
       </c>
       <c r="F424" t="n">
-        <v>0.14</v>
+        <v>0.1</v>
       </c>
       <c r="G424" t="inlineStr"/>
     </row>
@@ -13624,7 +13624,7 @@
         </is>
       </c>
       <c r="F426" t="n">
-        <v>0.11</v>
+        <v>0.06</v>
       </c>
       <c r="G426" t="inlineStr"/>
     </row>
@@ -13655,7 +13655,7 @@
         </is>
       </c>
       <c r="F427" t="n">
-        <v>0.25</v>
+        <v>0.16</v>
       </c>
       <c r="G427" t="inlineStr"/>
     </row>
@@ -13686,7 +13686,7 @@
         </is>
       </c>
       <c r="F428" t="n">
-        <v>0.24</v>
+        <v>0.23</v>
       </c>
       <c r="G428" t="inlineStr"/>
     </row>
@@ -13717,7 +13717,7 @@
         </is>
       </c>
       <c r="F429" t="n">
-        <v>0.1</v>
+        <v>0.18</v>
       </c>
       <c r="G429" t="inlineStr"/>
     </row>
@@ -13748,7 +13748,7 @@
         </is>
       </c>
       <c r="F430" t="n">
-        <v>0.18</v>
+        <v>0.15</v>
       </c>
       <c r="G430" t="inlineStr"/>
     </row>
@@ -13779,7 +13779,7 @@
         </is>
       </c>
       <c r="F431" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.14</v>
       </c>
       <c r="G431" t="inlineStr"/>
     </row>
@@ -13810,7 +13810,7 @@
         </is>
       </c>
       <c r="F432" t="n">
-        <v>0.24</v>
+        <v>0.11</v>
       </c>
       <c r="G432" t="inlineStr"/>
     </row>
@@ -13841,7 +13841,7 @@
         </is>
       </c>
       <c r="F433" t="n">
-        <v>0.12</v>
+        <v>0.13</v>
       </c>
       <c r="G433" t="inlineStr"/>
     </row>
@@ -13872,7 +13872,7 @@
         </is>
       </c>
       <c r="F434" t="n">
-        <v>0.25</v>
+        <v>0.08</v>
       </c>
       <c r="G434" t="inlineStr"/>
     </row>
@@ -13903,7 +13903,7 @@
         </is>
       </c>
       <c r="F435" t="n">
-        <v>0.18</v>
+        <v>0.15</v>
       </c>
       <c r="G435" t="inlineStr"/>
     </row>
@@ -13934,7 +13934,7 @@
         </is>
       </c>
       <c r="F436" t="n">
-        <v>0.15</v>
+        <v>0.09</v>
       </c>
       <c r="G436" t="inlineStr"/>
     </row>
@@ -13965,7 +13965,7 @@
         </is>
       </c>
       <c r="F437" t="n">
-        <v>0.14</v>
+        <v>0.09</v>
       </c>
       <c r="G437" t="inlineStr"/>
     </row>
@@ -13996,7 +13996,7 @@
         </is>
       </c>
       <c r="F438" t="n">
-        <v>0.13</v>
+        <v>0.2</v>
       </c>
       <c r="G438" t="inlineStr"/>
     </row>
@@ -14027,7 +14027,7 @@
         </is>
       </c>
       <c r="F439" t="n">
-        <v>0.24</v>
+        <v>0.15</v>
       </c>
       <c r="G439" t="inlineStr"/>
     </row>
@@ -14058,7 +14058,7 @@
         </is>
       </c>
       <c r="F440" t="n">
-        <v>0.05</v>
+        <v>0.23</v>
       </c>
       <c r="G440" t="inlineStr"/>
     </row>
@@ -14089,7 +14089,7 @@
         </is>
       </c>
       <c r="F441" t="n">
-        <v>0.17</v>
+        <v>0.16</v>
       </c>
       <c r="G441" t="inlineStr"/>
     </row>
@@ -14120,7 +14120,7 @@
         </is>
       </c>
       <c r="F442" t="n">
-        <v>0.19</v>
+        <v>0.12</v>
       </c>
       <c r="G442" t="inlineStr"/>
     </row>
@@ -14151,7 +14151,7 @@
         </is>
       </c>
       <c r="F443" t="n">
-        <v>0.05</v>
+        <v>0.24</v>
       </c>
       <c r="G443" t="inlineStr"/>
     </row>
@@ -14182,7 +14182,7 @@
         </is>
       </c>
       <c r="F444" t="n">
-        <v>0.24</v>
+        <v>0.1</v>
       </c>
       <c r="G444" t="inlineStr"/>
     </row>
@@ -14244,7 +14244,7 @@
         </is>
       </c>
       <c r="F446" t="n">
-        <v>0.19</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="G446" t="inlineStr"/>
     </row>
@@ -14275,7 +14275,7 @@
         </is>
       </c>
       <c r="F447" t="n">
-        <v>0.06</v>
+        <v>0.25</v>
       </c>
       <c r="G447" t="inlineStr"/>
     </row>
@@ -14306,7 +14306,7 @@
         </is>
       </c>
       <c r="F448" t="n">
-        <v>0.22</v>
+        <v>0.14</v>
       </c>
       <c r="G448" t="inlineStr"/>
     </row>
@@ -14337,7 +14337,7 @@
         </is>
       </c>
       <c r="F449" t="n">
-        <v>0.2</v>
+        <v>0.09</v>
       </c>
       <c r="G449" t="inlineStr"/>
     </row>
@@ -14399,7 +14399,7 @@
         </is>
       </c>
       <c r="F451" t="n">
-        <v>0.19</v>
+        <v>0.1</v>
       </c>
       <c r="G451" t="inlineStr"/>
     </row>
@@ -14430,7 +14430,7 @@
         </is>
       </c>
       <c r="F452" t="n">
-        <v>0.22</v>
+        <v>0.15</v>
       </c>
       <c r="G452" t="inlineStr"/>
     </row>
@@ -14461,7 +14461,7 @@
         </is>
       </c>
       <c r="F453" t="n">
-        <v>0.06</v>
+        <v>0.19</v>
       </c>
       <c r="G453" t="inlineStr"/>
     </row>
@@ -14492,7 +14492,7 @@
         </is>
       </c>
       <c r="F454" t="n">
-        <v>0.16</v>
+        <v>0.1</v>
       </c>
       <c r="G454" t="inlineStr"/>
     </row>
@@ -14523,7 +14523,7 @@
         </is>
       </c>
       <c r="F455" t="n">
-        <v>0.24</v>
+        <v>0.12</v>
       </c>
       <c r="G455" t="inlineStr"/>
     </row>
@@ -14554,7 +14554,7 @@
         </is>
       </c>
       <c r="F456" t="n">
-        <v>0.21</v>
+        <v>0.06</v>
       </c>
       <c r="G456" t="inlineStr"/>
     </row>
@@ -14585,7 +14585,7 @@
         </is>
       </c>
       <c r="F457" t="n">
-        <v>0.1</v>
+        <v>0.13</v>
       </c>
       <c r="G457" t="inlineStr"/>
     </row>
@@ -14616,7 +14616,7 @@
         </is>
       </c>
       <c r="F458" t="n">
-        <v>0.15</v>
+        <v>0.14</v>
       </c>
       <c r="G458" t="inlineStr"/>
     </row>
@@ -14647,7 +14647,7 @@
         </is>
       </c>
       <c r="F459" t="n">
-        <v>0.18</v>
+        <v>0.23</v>
       </c>
       <c r="G459" t="inlineStr"/>
     </row>
@@ -14678,7 +14678,7 @@
         </is>
       </c>
       <c r="F460" t="n">
-        <v>0.18</v>
+        <v>0.1</v>
       </c>
       <c r="G460" t="inlineStr"/>
     </row>
@@ -14709,7 +14709,7 @@
         </is>
       </c>
       <c r="F461" t="n">
-        <v>0.15</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="G461" t="inlineStr"/>
     </row>
@@ -14740,7 +14740,7 @@
         </is>
       </c>
       <c r="F462" t="n">
-        <v>0.2</v>
+        <v>0.13</v>
       </c>
       <c r="G462" t="inlineStr"/>
     </row>
@@ -14771,7 +14771,7 @@
         </is>
       </c>
       <c r="F463" t="n">
-        <v>0.18</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="G463" t="inlineStr"/>
     </row>
@@ -14802,7 +14802,7 @@
         </is>
       </c>
       <c r="F464" t="n">
-        <v>0.24</v>
+        <v>0.23</v>
       </c>
       <c r="G464" t="inlineStr"/>
     </row>
@@ -14833,7 +14833,7 @@
         </is>
       </c>
       <c r="F465" t="n">
-        <v>0.1</v>
+        <v>0.14</v>
       </c>
       <c r="G465" t="inlineStr"/>
     </row>
@@ -14864,7 +14864,7 @@
         </is>
       </c>
       <c r="F466" t="n">
-        <v>0.18</v>
+        <v>0.19</v>
       </c>
       <c r="G466" t="inlineStr"/>
     </row>
@@ -14926,7 +14926,7 @@
         </is>
       </c>
       <c r="F468" t="n">
-        <v>0.11</v>
+        <v>0.21</v>
       </c>
       <c r="G468" t="inlineStr"/>
     </row>
@@ -14957,7 +14957,7 @@
         </is>
       </c>
       <c r="F469" t="n">
-        <v>0.07000000000000001</v>
+        <v>0.05</v>
       </c>
       <c r="G469" t="inlineStr"/>
     </row>
@@ -14988,7 +14988,7 @@
         </is>
       </c>
       <c r="F470" t="n">
-        <v>0.23</v>
+        <v>0.1</v>
       </c>
       <c r="G470" t="inlineStr"/>
     </row>
@@ -15019,7 +15019,7 @@
         </is>
       </c>
       <c r="F471" t="n">
-        <v>0.09</v>
+        <v>0.15</v>
       </c>
       <c r="G471" t="inlineStr"/>
     </row>

</xml_diff>